<commit_message>
Restore the Pareto input headers the ranked block had blanked
header() writes every column in the row, so adding the ranked block's headers
through it wrote empty strings over A4:E4 and left 57 input cells sitting under
a blank header. The ranked block writes its own five cells now.
</commit_message>
<xml_diff>
--- a/templates/25-pareto-and-distribution.xlsx
+++ b/templates/25-pareto-and-distribution.xlsx
@@ -909,12 +909,31 @@
       <c r="K3" s="7" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr"/>
-      <c r="B4" s="8" t="inlineStr"/>
-      <c r="C4" s="8" t="inlineStr"/>
-      <c r="D4" s="8" t="inlineStr"/>
-      <c r="E4" s="8" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Validated by reading tickets?</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
           <t>#</t>

</xml_diff>